<commit_message>
custom common validate date and allow null condtion for external quality report
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ImportTapeEnRouteTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ImportTapeEnRouteTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\i_phong.nv_3si\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Tháng đặt hàng</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>O.P Dlv DT</t>
+  </si>
+  <si>
+    <t>Transmit</t>
   </si>
 </sst>
 </file>
@@ -158,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -184,6 +187,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultColWidth="18.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" style="8"/>
@@ -474,13 +481,14 @@
     <col min="8" max="8" width="18.140625" style="8"/>
     <col min="9" max="11" width="18.140625" style="1"/>
     <col min="12" max="12" width="18.140625" style="10"/>
-    <col min="13" max="13" width="18.140625" style="8"/>
-    <col min="14" max="15" width="18.140625" style="10"/>
-    <col min="16" max="16" width="18.140625" style="8"/>
-    <col min="17" max="16384" width="18.140625" style="1"/>
+    <col min="13" max="13" width="18.140625" style="12"/>
+    <col min="14" max="14" width="18.140625" style="8"/>
+    <col min="15" max="16" width="18.140625" style="10"/>
+    <col min="17" max="17" width="18.140625" style="8"/>
+    <col min="18" max="16384" width="18.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="7" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="7" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -517,16 +525,19 @@
       <c r="L1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix template import tape
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ImportTapeEnRouteTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ImportTapeEnRouteTemplate.xlsx
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -191,6 +191,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr defaultColWidth="18.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" style="8"/>
@@ -485,61 +488,66 @@
     <col min="14" max="14" width="18.140625" style="8"/>
     <col min="15" max="16" width="18.140625" style="10"/>
     <col min="17" max="17" width="18.140625" style="8"/>
-    <col min="18" max="16384" width="18.140625" style="1"/>
+    <col min="18" max="18" width="37.42578125" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="18.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="7" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:33" s="13" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:33" s="7" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>13</v>
       </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="AG3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>